<commit_message>
Rev A errors identified in spreadsheet
</commit_message>
<xml_diff>
--- a/Karman Delta Arm/Assembly Outputs/Bill of Materials/KDA Rev A1 PCB BOM.xlsx
+++ b/Karman Delta Arm/Assembly Outputs/Bill of Materials/KDA Rev A1 PCB BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adria\Documents\GitHub\AltiumGithub\Karman Delta Arm\Assembly Outputs\Bill of Materials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{454DB966-A9F3-4E0F-A06E-7431644F33BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B7B08D8-44AC-4EB2-9BE4-A545A36F1011}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33825" yWindow="3630" windowWidth="32160" windowHeight="16740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="29010" windowHeight="16740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PCB BOM" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="174">
   <si>
     <t>Item #</t>
   </si>
@@ -442,7 +442,7 @@
     <t>KDA Rev A</t>
   </si>
   <si>
-    <t>77-VJ0603Y104KXACWBC</t>
+    <t>2407338</t>
   </si>
   <si>
     <t>3013414</t>
@@ -511,7 +511,7 @@
     <t>952-1478-1-ND</t>
   </si>
   <si>
-    <t>8000564</t>
+    <t>2250281</t>
   </si>
   <si>
     <t>2301278</t>
@@ -520,7 +520,7 @@
     <t>296-32484-1-ND</t>
   </si>
   <si>
-    <t>998-MIC5200-3.3YSTR</t>
+    <t>2851609</t>
   </si>
   <si>
     <t>296-53076-ND</t>
@@ -532,24 +532,18 @@
     <t>2770298</t>
   </si>
   <si>
-    <t>WM11300-ND</t>
+    <t>3726670</t>
   </si>
   <si>
     <t>Supplier 1</t>
   </si>
   <si>
-    <t>Mouser</t>
-  </si>
-  <si>
     <t>Farnell</t>
   </si>
   <si>
     <t>DigiKey</t>
   </si>
   <si>
-    <t>Future Electronics</t>
-  </si>
-  <si>
     <t>Fitted</t>
   </si>
   <si>
@@ -560,6 +554,12 @@
   </si>
   <si>
     <t>7 Nov 2025</t>
+  </si>
+  <si>
+    <t>Qty</t>
+  </si>
+  <si>
+    <t>Buy Qty</t>
   </si>
 </sst>
 </file>
@@ -737,14 +737,14 @@
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1104,7 +1104,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:J167"/>
+  <dimension ref="A1:K167"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.5703125" style="1" bestFit="1" customWidth="1"/>
@@ -1119,44 +1119,44 @@
     <col min="12" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B1" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="29" t="s">
+      <c r="C1" s="27" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B2" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="29" t="s">
+      <c r="C2" s="27" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="27" t="s">
+      <c r="D2" s="29" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
       <c r="I2" s="7"/>
     </row>
-    <row r="3" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B3" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="29" t="s">
+      <c r="C3" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="28"/>
-      <c r="E3" s="28"/>
-      <c r="F3" s="28"/>
-      <c r="G3" s="28"/>
-      <c r="H3" s="28"/>
-    </row>
-    <row r="4" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="30"/>
+      <c r="G3" s="30"/>
+      <c r="H3" s="30"/>
+    </row>
+    <row r="4" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B4" s="10" t="s">
         <v>1</v>
       </c>
@@ -1164,60 +1164,66 @@
         <f>Parameters!A3</f>
         <v>7 Nov 2025</v>
       </c>
-      <c r="D4" s="28"/>
-      <c r="E4" s="28"/>
-      <c r="F4" s="28"/>
-      <c r="G4" s="28"/>
-      <c r="H4" s="28"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="30"/>
+      <c r="F4" s="30"/>
+      <c r="G4" s="30"/>
+      <c r="H4" s="30"/>
       <c r="I4" s="8"/>
     </row>
-    <row r="5" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="29" t="s">
+      <c r="C5" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="28"/>
-      <c r="E5" s="28"/>
-      <c r="F5" s="28"/>
-      <c r="G5" s="28"/>
-      <c r="H5" s="28"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
       <c r="I5" s="8"/>
     </row>
-    <row r="6" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="29" t="s">
+      <c r="C6" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="28"/>
-      <c r="E6" s="28"/>
-      <c r="F6" s="28"/>
-      <c r="G6" s="28"/>
-      <c r="H6" s="28"/>
+      <c r="D6" s="30"/>
+      <c r="E6" s="30"/>
+      <c r="F6" s="30"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="30"/>
       <c r="I6" s="4"/>
     </row>
-    <row r="7" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
-      <c r="D7" s="28"/>
-      <c r="E7" s="28"/>
-      <c r="F7" s="28"/>
-      <c r="G7" s="28"/>
-      <c r="H7" s="28"/>
+      <c r="D7" s="30"/>
+      <c r="E7" s="30"/>
+      <c r="F7" s="30"/>
+      <c r="G7" s="30"/>
+      <c r="H7" s="30"/>
       <c r="I7" s="4"/>
-    </row>
-    <row r="8" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K7" s="1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C8" s="4"/>
       <c r="D8" s="13"/>
       <c r="E8" s="13"/>
       <c r="F8" s="13"/>
       <c r="G8" s="13"/>
       <c r="H8" s="13"/>
-    </row>
-    <row r="9" spans="1:10" s="21" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="K8" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" s="21" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A9" s="20" t="s">
         <v>0</v>
       </c>
@@ -1243,15 +1249,18 @@
         <v>165</v>
       </c>
       <c r="I9" s="20" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J9" s="20" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
+        <v>169</v>
+      </c>
+      <c r="K9" s="21" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A10" s="22">
-        <f>ROW(A10) - ROW($A$9)</f>
+        <f t="shared" ref="A10:A41" si="0">ROW(A10) - ROW($A$9)</f>
         <v>1</v>
       </c>
       <c r="B10" s="5" t="s">
@@ -1270,15 +1279,19 @@
       </c>
       <c r="H10" s="16"/>
       <c r="I10" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="J10" s="24" t="s">
         <v>170</v>
       </c>
-      <c r="J10" s="24" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="89.25" x14ac:dyDescent="0.2">
+      <c r="K10" s="12">
+        <f>D10*$K$8</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="89.25" x14ac:dyDescent="0.2">
       <c r="A11" s="25">
-        <f>ROW(A11) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="B11" s="6" t="s">
@@ -1303,13 +1316,17 @@
         <v>166</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J11" s="24"/>
-    </row>
-    <row r="12" spans="1:10" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="K11" s="12">
+        <f t="shared" ref="K11:K42" si="1">D11*$K$8</f>
+        <v>155</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A12" s="22">
-        <f>ROW(A12) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>3</v>
       </c>
       <c r="B12" s="5" t="s">
@@ -1331,16 +1348,20 @@
         <v>135</v>
       </c>
       <c r="H12" s="16" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J12" s="24"/>
-    </row>
-    <row r="13" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="K12" s="12">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A13" s="25">
-        <f>ROW(A13) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="B13" s="6" t="s">
@@ -1362,16 +1383,20 @@
         <v>136</v>
       </c>
       <c r="H13" s="17" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J13" s="24"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K13" s="12">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A14" s="22">
-        <f>ROW(A14) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="B14" s="5" t="s">
@@ -1393,16 +1418,20 @@
         <v>137</v>
       </c>
       <c r="H14" s="16" t="s">
+        <v>167</v>
+      </c>
+      <c r="I14" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="I14" s="6" t="s">
-        <v>170</v>
-      </c>
       <c r="J14" s="24"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K14" s="12">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A15" s="25">
-        <f>ROW(A15) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="B15" s="6" t="s">
@@ -1424,16 +1453,20 @@
         <v>138</v>
       </c>
       <c r="H15" s="17" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J15" s="24"/>
-    </row>
-    <row r="16" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="K15" s="12">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A16" s="22">
-        <f>ROW(A16) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
       <c r="B16" s="5" t="s">
@@ -1455,16 +1488,20 @@
         <v>139</v>
       </c>
       <c r="H16" s="16" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J16" s="24"/>
-    </row>
-    <row r="17" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="K16" s="12">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A17" s="25">
-        <f>ROW(A17) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="B17" s="6" t="s">
@@ -1486,16 +1523,20 @@
         <v>140</v>
       </c>
       <c r="H17" s="17" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J17" s="24"/>
-    </row>
-    <row r="18" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="K17" s="12">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A18" s="22">
-        <f>ROW(A18) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="B18" s="5" t="s">
@@ -1517,16 +1558,20 @@
         <v>141</v>
       </c>
       <c r="H18" s="16" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J18" s="24"/>
-    </row>
-    <row r="19" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="K18" s="12">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A19" s="25">
-        <f>ROW(A19) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="B19" s="6" t="s">
@@ -1548,16 +1593,20 @@
         <v>142</v>
       </c>
       <c r="H19" s="17" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I19" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J19" s="24"/>
-    </row>
-    <row r="20" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="K19" s="12">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A20" s="22">
-        <f>ROW(A20) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>11</v>
       </c>
       <c r="B20" s="5" t="s">
@@ -1579,16 +1628,20 @@
         <v>143</v>
       </c>
       <c r="H20" s="16" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I20" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J20" s="24"/>
-    </row>
-    <row r="21" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="K20" s="12">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A21" s="25">
-        <f>ROW(A21) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="B21" s="6" t="s">
@@ -1610,16 +1663,20 @@
         <v>144</v>
       </c>
       <c r="H21" s="17" t="s">
+        <v>167</v>
+      </c>
+      <c r="I21" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="I21" s="6" t="s">
-        <v>170</v>
-      </c>
       <c r="J21" s="24"/>
-    </row>
-    <row r="22" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="K21" s="12">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A22" s="22">
-        <f>ROW(A22) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
       <c r="B22" s="5" t="s">
@@ -1641,16 +1698,20 @@
         <v>145</v>
       </c>
       <c r="H22" s="16" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I22" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J22" s="24"/>
-    </row>
-    <row r="23" spans="1:10" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="K22" s="12">
+        <f t="shared" si="1"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="38.25" x14ac:dyDescent="0.2">
       <c r="A23" s="25">
-        <f>ROW(A23) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="B23" s="6" t="s">
@@ -1672,16 +1733,20 @@
         <v>146</v>
       </c>
       <c r="H23" s="17" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I23" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J23" s="24"/>
-    </row>
-    <row r="24" spans="1:10" ht="51" x14ac:dyDescent="0.2">
+      <c r="K23" s="12">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="51" x14ac:dyDescent="0.2">
       <c r="A24" s="22">
-        <f>ROW(A24) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
       <c r="B24" s="5" t="s">
@@ -1703,16 +1768,20 @@
         <v>147</v>
       </c>
       <c r="H24" s="16" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I24" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J24" s="24"/>
-    </row>
-    <row r="25" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="K24" s="12">
+        <f t="shared" si="1"/>
+        <v>85</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A25" s="25">
-        <f>ROW(A25) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="B25" s="6" t="s">
@@ -1734,16 +1803,20 @@
         <v>148</v>
       </c>
       <c r="H25" s="17" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I25" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J25" s="24"/>
-    </row>
-    <row r="26" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="K25" s="12">
+        <f t="shared" si="1"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A26" s="22">
-        <f>ROW(A26) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>17</v>
       </c>
       <c r="B26" s="5" t="s">
@@ -1765,16 +1838,20 @@
         <v>149</v>
       </c>
       <c r="H26" s="16" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I26" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J26" s="24"/>
-    </row>
-    <row r="27" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="K26" s="12">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A27" s="25">
-        <f>ROW(A27) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="B27" s="6" t="s">
@@ -1796,16 +1873,20 @@
         <v>150</v>
       </c>
       <c r="H27" s="17" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I27" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J27" s="24"/>
-    </row>
-    <row r="28" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="K27" s="12">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A28" s="22">
-        <f>ROW(A28) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>19</v>
       </c>
       <c r="B28" s="5" t="s">
@@ -1827,16 +1908,20 @@
         <v>151</v>
       </c>
       <c r="H28" s="16" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I28" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J28" s="24"/>
-    </row>
-    <row r="29" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="K28" s="12">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A29" s="25">
-        <f>ROW(A29) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="B29" s="6" t="s">
@@ -1858,16 +1943,20 @@
         <v>152</v>
       </c>
       <c r="H29" s="17" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I29" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J29" s="24"/>
-    </row>
-    <row r="30" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="K29" s="12">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A30" s="22">
-        <f>ROW(A30) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="B30" s="5" t="s">
@@ -1889,16 +1978,20 @@
         <v>153</v>
       </c>
       <c r="H30" s="16" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I30" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J30" s="24"/>
-    </row>
-    <row r="31" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="K30" s="12">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A31" s="25">
-        <f>ROW(A31) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="B31" s="6" t="s">
@@ -1920,16 +2013,20 @@
         <v>154</v>
       </c>
       <c r="H31" s="17" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I31" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J31" s="24"/>
-    </row>
-    <row r="32" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="K31" s="12">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A32" s="22">
-        <f>ROW(A32) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="B32" s="5" t="s">
@@ -1951,16 +2048,20 @@
         <v>155</v>
       </c>
       <c r="H32" s="16" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I32" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J32" s="24"/>
-    </row>
-    <row r="33" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="K32" s="12">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A33" s="25">
-        <f>ROW(A33) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>24</v>
       </c>
       <c r="B33" s="6" t="s">
@@ -1982,16 +2083,20 @@
         <v>156</v>
       </c>
       <c r="H33" s="17" t="s">
+        <v>167</v>
+      </c>
+      <c r="I33" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="I33" s="6" t="s">
-        <v>170</v>
-      </c>
       <c r="J33" s="24"/>
-    </row>
-    <row r="34" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="K33" s="12">
+        <f t="shared" si="1"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A34" s="22">
-        <f>ROW(A34) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>25</v>
       </c>
       <c r="B34" s="5" t="s">
@@ -2013,16 +2118,20 @@
         <v>157</v>
       </c>
       <c r="H34" s="16" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="I34" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J34" s="24"/>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K34" s="12">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35" s="25">
-        <f>ROW(A35) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>26</v>
       </c>
       <c r="B35" s="6" t="s">
@@ -2044,16 +2153,20 @@
         <v>158</v>
       </c>
       <c r="H35" s="17" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I35" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J35" s="24"/>
-    </row>
-    <row r="36" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="K35" s="12">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A36" s="22">
-        <f>ROW(A36) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>27</v>
       </c>
       <c r="B36" s="5" t="s">
@@ -2075,16 +2188,20 @@
         <v>159</v>
       </c>
       <c r="H36" s="16" t="s">
+        <v>167</v>
+      </c>
+      <c r="I36" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="I36" s="6" t="s">
-        <v>170</v>
-      </c>
       <c r="J36" s="24"/>
-    </row>
-    <row r="37" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="K36" s="12">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A37" s="25">
-        <f>ROW(A37) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>28</v>
       </c>
       <c r="B37" s="6" t="s">
@@ -2109,13 +2226,17 @@
         <v>166</v>
       </c>
       <c r="I37" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J37" s="24"/>
-    </row>
-    <row r="38" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="K37" s="12">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A38" s="22">
-        <f>ROW(A38) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>29</v>
       </c>
       <c r="B38" s="5" t="s">
@@ -2137,16 +2258,20 @@
         <v>161</v>
       </c>
       <c r="H38" s="16" t="s">
+        <v>167</v>
+      </c>
+      <c r="I38" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="I38" s="6" t="s">
-        <v>170</v>
-      </c>
       <c r="J38" s="24"/>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K38" s="12">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A39" s="25">
-        <f>ROW(A39) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>30</v>
       </c>
       <c r="B39" s="6" t="s">
@@ -2168,16 +2293,20 @@
         <v>162</v>
       </c>
       <c r="H39" s="17" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I39" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J39" s="24"/>
-    </row>
-    <row r="40" spans="1:10" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="K39" s="12">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="25.5" x14ac:dyDescent="0.2">
       <c r="A40" s="22">
-        <f>ROW(A40) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>31</v>
       </c>
       <c r="B40" s="5" t="s">
@@ -2199,16 +2328,20 @@
         <v>163</v>
       </c>
       <c r="H40" s="16" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="I40" s="6" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="J40" s="24"/>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="K40" s="12">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A41" s="25">
-        <f>ROW(A41) - ROW($A$9)</f>
+        <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="B41" s="6" t="s">
@@ -2230,14 +2363,18 @@
         <v>164</v>
       </c>
       <c r="H41" s="17" t="s">
+        <v>166</v>
+      </c>
+      <c r="I41" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="I41" s="6" t="s">
-        <v>170</v>
-      </c>
       <c r="J41" s="24"/>
-    </row>
-    <row r="42" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K41" s="12">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B42" s="2"/>
       <c r="C42" s="3"/>
       <c r="D42" s="18"/>
@@ -2246,8 +2383,9 @@
       <c r="G42" s="14"/>
       <c r="H42" s="18"/>
       <c r="I42" s="3"/>
-    </row>
-    <row r="43" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="K42" s="12"/>
+    </row>
+    <row r="43" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B43" s="2"/>
       <c r="C43" s="3"/>
       <c r="D43" s="18"/>
@@ -2257,7 +2395,7 @@
       <c r="H43" s="18"/>
       <c r="I43" s="3"/>
     </row>
-    <row r="44" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B44" s="2"/>
       <c r="C44" s="3"/>
       <c r="D44" s="18"/>
@@ -2267,7 +2405,7 @@
       <c r="H44" s="18"/>
       <c r="I44" s="3"/>
     </row>
-    <row r="45" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B45" s="2"/>
       <c r="C45" s="3"/>
       <c r="D45" s="18"/>
@@ -2277,7 +2415,7 @@
       <c r="H45" s="18"/>
       <c r="I45" s="3"/>
     </row>
-    <row r="46" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:11" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B46" s="2"/>
       <c r="C46" s="3"/>
       <c r="D46" s="18"/>
@@ -2287,7 +2425,7 @@
       <c r="H46" s="18"/>
       <c r="I46" s="3"/>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B47" s="2"/>
       <c r="C47" s="3"/>
       <c r="D47" s="18"/>
@@ -2297,7 +2435,7 @@
       <c r="H47" s="18"/>
       <c r="I47" s="3"/>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.2">
       <c r="B48" s="2"/>
       <c r="C48" s="3"/>
       <c r="D48" s="18"/>
@@ -3514,13 +3652,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="30" t="s">
-        <v>173</v>
+      <c r="A1" s="28" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="30" t="s">
-        <v>173</v>
+      <c r="A2" s="28" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>